<commit_message>
feat: rev1 initial (diagrams & sales asco)
</commit_message>
<xml_diff>
--- a/BT_Use_Case_Description.xlsx
+++ b/BT_Use_Case_Description.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ASLAB\TPA\DESKTOP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F6D8479-9F58-4008-8095-6A19681BFEC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{534CB5E1-54B4-4A8A-A457-88E0B102F103}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="599" activeTab="1" xr2:uid="{2183EE87-2FE0-1848-A8EC-EAF6DA5552F2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="599" firstSheet="4" activeTab="4" xr2:uid="{2183EE87-2FE0-1848-A8EC-EAF6DA5552F2}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Allocate Chef and Waiter" sheetId="1" r:id="rId1"/>
@@ -268,9 +268,6 @@
     <t>Propose Store Removal</t>
   </si>
   <si>
-    <t>View All Store Details</t>
-  </si>
-  <si>
     <t>Retail Manager</t>
   </si>
   <si>
@@ -338,16 +335,6 @@
     <t>1.1 Display all store list</t>
   </si>
   <si>
-    <t>3. Retail Manager will choose a souvenir to remove</t>
-  </si>
-  <si>
-    <t>3.1 Update the store data in the database</t>
-  </si>
-  <si>
-    <t>3.2 Generate a success message confirming the removal of 
-a souvenir from the store</t>
-  </si>
-  <si>
     <t>4. Retail Manager receive a success message</t>
   </si>
   <si>
@@ -547,6 +534,19 @@
   </si>
   <si>
     <t>3.1 Validate form fields must not be empty except finder and image if status if 'missing'</t>
+  </si>
+  <si>
+    <t>2.1 Update the store data in the database</t>
+  </si>
+  <si>
+    <t>2.2 Generate a success message confirming the removal of 
+a souvenir from the store</t>
+  </si>
+  <si>
+    <t>2. Retail Manager will choose a souvenir to remove</t>
+  </si>
+  <si>
+    <t>3. Retail Manager receive a success message</t>
   </si>
 </sst>
 </file>
@@ -758,6 +758,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -785,57 +794,60 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -843,18 +855,6 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
@@ -1183,85 +1183,85 @@
       <c r="B2" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="30" t="s">
+      <c r="C2" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="31"/>
+      <c r="D2" s="20"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B3" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="D3" s="19"/>
+      <c r="D3" s="22"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="D4" s="19"/>
+      <c r="D4" s="22"/>
     </row>
     <row r="5" spans="2:4" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="28" t="s">
+      <c r="C5" s="30" t="s">
         <v>56</v>
       </c>
-      <c r="D5" s="29"/>
+      <c r="D5" s="31"/>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B6" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="19"/>
+      <c r="D6" s="22"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B7" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="19"/>
+      <c r="D7" s="22"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B8" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="18" t="s">
-        <v>107</v>
-      </c>
-      <c r="D8" s="19"/>
+      <c r="C8" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="D8" s="22"/>
     </row>
     <row r="9" spans="2:4" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="28" t="s">
+      <c r="C9" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="29"/>
+      <c r="D9" s="31"/>
     </row>
     <row r="10" spans="2:4" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="28" t="s">
+      <c r="C10" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="D10" s="19"/>
+      <c r="D10" s="22"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B11" s="20" t="s">
+      <c r="B11" s="23" t="s">
         <v>9</v>
       </c>
       <c r="C11" s="13" t="s">
@@ -1272,7 +1272,7 @@
       </c>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B12" s="21"/>
+      <c r="B12" s="24"/>
       <c r="C12" s="2" t="s">
         <v>18</v>
       </c>
@@ -1281,8 +1281,8 @@
       </c>
     </row>
     <row r="13" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="21"/>
-      <c r="C13" s="25" t="s">
+      <c r="B13" s="24"/>
+      <c r="C13" s="28" t="s">
         <v>37</v>
       </c>
       <c r="D13" s="2" t="s">
@@ -1290,87 +1290,81 @@
       </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B14" s="21"/>
-      <c r="C14" s="26"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="29"/>
       <c r="D14" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B15" s="21"/>
-      <c r="C15" s="26"/>
+      <c r="B15" s="24"/>
+      <c r="C15" s="29"/>
       <c r="D15" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B16" s="24"/>
+      <c r="C16" s="32"/>
+      <c r="D16" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B17" s="24"/>
+      <c r="C17" s="28" t="s">
+        <v>114</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B18" s="24"/>
+      <c r="C18" s="29"/>
+      <c r="D18" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="24"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="4" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B16" s="21"/>
-      <c r="C16" s="27"/>
-      <c r="D16" s="2" t="s">
+    <row r="20" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B20" s="25"/>
+      <c r="C20" s="4" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B17" s="21"/>
-      <c r="C17" s="25" t="s">
-        <v>118</v>
-      </c>
-      <c r="D17" s="2" t="s">
+      <c r="D20" s="3"/>
+    </row>
+    <row r="21" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B21" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="D21" s="22"/>
+    </row>
+    <row r="22" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B22" s="24"/>
+      <c r="C22" s="26" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B18" s="21"/>
-      <c r="C18" s="26"/>
-      <c r="D18" s="2" t="s">
+      <c r="D22" s="27"/>
+    </row>
+    <row r="23" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B23" s="25"/>
+      <c r="C23" s="7" t="s">
         <v>122</v>
-      </c>
-    </row>
-    <row r="19" spans="2:4" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="21"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="4" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B20" s="22"/>
-      <c r="C20" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="D20" s="3"/>
-    </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B21" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="C21" s="18" t="s">
-        <v>28</v>
-      </c>
-      <c r="D21" s="19"/>
-    </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B22" s="21"/>
-      <c r="C22" s="23" t="s">
-        <v>125</v>
-      </c>
-      <c r="D22" s="24"/>
-    </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B23" s="22"/>
-      <c r="C23" s="7" t="s">
-        <v>126</v>
       </c>
       <c r="D23" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="C4:D4"/>
     <mergeCell ref="B21:B23"/>
     <mergeCell ref="C22:D22"/>
     <mergeCell ref="C17:C19"/>
@@ -1380,6 +1374,12 @@
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="C21:D21"/>
     <mergeCell ref="C13:C16"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="C4:D4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1399,85 +1399,85 @@
       <c r="B2" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="30" t="s">
+      <c r="C2" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="D2" s="31"/>
+      <c r="D2" s="20"/>
     </row>
     <row r="3" spans="2:4" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="28" t="s">
+      <c r="C3" s="30" t="s">
         <v>54</v>
       </c>
-      <c r="D3" s="29"/>
+      <c r="D3" s="31"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="D4" s="19"/>
+      <c r="D4" s="22"/>
     </row>
     <row r="5" spans="2:4" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="28" t="s">
+      <c r="C5" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="D5" s="29"/>
+      <c r="D5" s="31"/>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B6" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="19"/>
+      <c r="D6" s="22"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B7" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="19"/>
+      <c r="D7" s="22"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B8" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="18" t="s">
-        <v>87</v>
-      </c>
-      <c r="D8" s="19"/>
+      <c r="C8" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D8" s="22"/>
     </row>
     <row r="9" spans="2:4" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="43" t="s">
+      <c r="C9" s="33" t="s">
         <v>49</v>
       </c>
-      <c r="D9" s="43"/>
+      <c r="D9" s="33"/>
     </row>
     <row r="10" spans="2:4" ht="31.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="43" t="s">
+      <c r="C10" s="33" t="s">
         <v>58</v>
       </c>
-      <c r="D10" s="32"/>
+      <c r="D10" s="34"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B11" s="20" t="s">
+      <c r="B11" s="23" t="s">
         <v>9</v>
       </c>
       <c r="C11" s="13" t="s">
@@ -1488,7 +1488,7 @@
       </c>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B12" s="21"/>
+      <c r="B12" s="24"/>
       <c r="C12" s="2" t="s">
         <v>25</v>
       </c>
@@ -1497,8 +1497,8 @@
       </c>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B13" s="21"/>
-      <c r="C13" s="43" t="s">
+      <c r="B13" s="24"/>
+      <c r="C13" s="33" t="s">
         <v>26</v>
       </c>
       <c r="D13" s="2" t="s">
@@ -1506,46 +1506,46 @@
       </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B14" s="21"/>
-      <c r="C14" s="43"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="33"/>
       <c r="D14" s="3" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="21"/>
-      <c r="C15" s="43"/>
+      <c r="B15" s="24"/>
+      <c r="C15" s="33"/>
       <c r="D15" s="2" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="24"/>
+      <c r="C16" s="28" t="s">
+        <v>124</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B17" s="24"/>
+      <c r="C17" s="29"/>
+      <c r="D17" s="2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="B18" s="24"/>
+      <c r="C18" s="32"/>
+      <c r="D18" s="4" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B19" s="25"/>
+      <c r="C19" s="2" t="s">
         <v>127</v>
-      </c>
-    </row>
-    <row r="16" spans="2:4" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="21"/>
-      <c r="C16" s="25" t="s">
-        <v>128</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B17" s="21"/>
-      <c r="C17" s="26"/>
-      <c r="D17" s="2" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="18" spans="2:4" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B18" s="21"/>
-      <c r="C18" s="27"/>
-      <c r="D18" s="4" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B19" s="22"/>
-      <c r="C19" s="2" t="s">
-        <v>131</v>
       </c>
       <c r="D19" s="2"/>
     </row>
@@ -1561,7 +1561,7 @@
     <row r="21" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B21" s="9"/>
       <c r="C21" s="14" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="D21" s="3"/>
     </row>
@@ -1598,85 +1598,85 @@
       <c r="B2" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="37" t="s">
+      <c r="C2" s="35" t="s">
         <v>31</v>
       </c>
-      <c r="D2" s="38"/>
+      <c r="D2" s="36"/>
     </row>
     <row r="3" spans="2:4" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="28" t="s">
+      <c r="C3" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="D3" s="29"/>
+      <c r="D3" s="31"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="23" t="s">
+      <c r="C4" s="26" t="s">
         <v>34</v>
       </c>
-      <c r="D4" s="24"/>
+      <c r="D4" s="27"/>
     </row>
     <row r="5" spans="2:4" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="28" t="s">
+      <c r="C5" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="D5" s="29"/>
+      <c r="D5" s="31"/>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B6" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="23" t="s">
+      <c r="C6" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="24"/>
+      <c r="D6" s="27"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B7" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="23" t="s">
+      <c r="C7" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="24"/>
+      <c r="D7" s="27"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B8" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="23" t="s">
+      <c r="C8" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="24"/>
+      <c r="D8" s="27"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B9" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="28" t="s">
+      <c r="C9" s="30" t="s">
         <v>50</v>
       </c>
-      <c r="D9" s="29"/>
+      <c r="D9" s="31"/>
     </row>
     <row r="10" spans="2:4" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="28" t="s">
+      <c r="C10" s="30" t="s">
         <v>59</v>
       </c>
-      <c r="D10" s="19"/>
+      <c r="D10" s="22"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B11" s="34" t="s">
+      <c r="B11" s="37" t="s">
         <v>9</v>
       </c>
       <c r="C11" s="1" t="s">
@@ -1687,7 +1687,7 @@
       </c>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B12" s="35"/>
+      <c r="B12" s="38"/>
       <c r="C12" s="2" t="s">
         <v>38</v>
       </c>
@@ -1696,30 +1696,30 @@
       </c>
     </row>
     <row r="13" spans="2:4" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="35"/>
-      <c r="C13" s="25" t="s">
-        <v>116</v>
+      <c r="B13" s="38"/>
+      <c r="C13" s="28" t="s">
+        <v>112</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B14" s="35"/>
-      <c r="C14" s="26"/>
+      <c r="B14" s="38"/>
+      <c r="C14" s="29"/>
       <c r="D14" s="2" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B15" s="35"/>
-      <c r="C15" s="27"/>
+      <c r="B15" s="38"/>
+      <c r="C15" s="32"/>
       <c r="D15" s="4" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B16" s="36"/>
+      <c r="B16" s="39"/>
       <c r="C16" s="4" t="s">
         <v>43</v>
       </c>
@@ -1729,13 +1729,14 @@
       <c r="B17" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="23" t="s">
+      <c r="C17" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="D17" s="24"/>
+      <c r="D17" s="27"/>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B11:B16"/>
     <mergeCell ref="C17:D17"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="C3:D3"/>
@@ -1747,7 +1748,6 @@
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="C10:D10"/>
-    <mergeCell ref="B11:B16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1767,85 +1767,85 @@
       <c r="B2" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="37" t="s">
+      <c r="C2" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="D2" s="38"/>
+      <c r="D2" s="36"/>
     </row>
     <row r="3" spans="2:4" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="28" t="s">
+      <c r="C3" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="D3" s="29"/>
+      <c r="D3" s="31"/>
     </row>
     <row r="4" spans="2:4" ht="31.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="28" t="s">
+      <c r="C4" s="30" t="s">
         <v>52</v>
       </c>
-      <c r="D4" s="19"/>
+      <c r="D4" s="22"/>
     </row>
     <row r="5" spans="2:4" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="28" t="s">
+      <c r="C5" s="30" t="s">
         <v>57</v>
       </c>
-      <c r="D5" s="29"/>
+      <c r="D5" s="31"/>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B6" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="23" t="s">
+      <c r="C6" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="D6" s="24"/>
+      <c r="D6" s="27"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B7" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="23" t="s">
+      <c r="C7" s="26" t="s">
         <v>48</v>
       </c>
-      <c r="D7" s="24"/>
+      <c r="D7" s="27"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B8" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="23" t="s">
+      <c r="C8" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="D8" s="24"/>
+      <c r="D8" s="27"/>
     </row>
     <row r="9" spans="2:4" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="28" t="s">
+      <c r="C9" s="30" t="s">
         <v>51</v>
       </c>
-      <c r="D9" s="29"/>
+      <c r="D9" s="31"/>
     </row>
     <row r="10" spans="2:4" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="28" t="s">
+      <c r="C10" s="30" t="s">
         <v>60</v>
       </c>
-      <c r="D10" s="19"/>
+      <c r="D10" s="22"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B11" s="33" t="s">
+      <c r="B11" s="43" t="s">
         <v>9</v>
       </c>
       <c r="C11" s="5" t="s">
@@ -1856,7 +1856,7 @@
       </c>
     </row>
     <row r="12" spans="2:4" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B12" s="33"/>
+      <c r="B12" s="43"/>
       <c r="C12" s="17" t="s">
         <v>61</v>
       </c>
@@ -1865,8 +1865,8 @@
       </c>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B13" s="33"/>
-      <c r="C13" s="25" t="s">
+      <c r="B13" s="43"/>
+      <c r="C13" s="28" t="s">
         <v>65</v>
       </c>
       <c r="D13" s="2" t="s">
@@ -1874,81 +1874,88 @@
       </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B14" s="33"/>
-      <c r="C14" s="26"/>
+      <c r="B14" s="43"/>
+      <c r="C14" s="29"/>
       <c r="D14" s="3" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="33"/>
-      <c r="C15" s="27"/>
+      <c r="B15" s="43"/>
+      <c r="C15" s="32"/>
       <c r="D15" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="43"/>
+      <c r="C16" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B17" s="43"/>
+      <c r="C17" s="41"/>
+      <c r="D17" s="16" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B18" s="43"/>
+      <c r="C18" s="41"/>
+      <c r="D18" s="2" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="B19" s="43"/>
+      <c r="C19" s="42"/>
+      <c r="D19" s="4" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B20" s="43"/>
+      <c r="C20" s="15" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="16" spans="2:4" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="33"/>
-      <c r="C16" s="39" t="s">
-        <v>132</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B17" s="33"/>
-      <c r="C17" s="40"/>
-      <c r="D17" s="16" t="s">
+      <c r="D20" s="2"/>
+    </row>
+    <row r="21" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B21" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="D21" s="22"/>
+    </row>
+    <row r="22" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B22" s="24"/>
+      <c r="C22" s="21" t="s">
+        <v>122</v>
+      </c>
+      <c r="D22" s="22"/>
+    </row>
+    <row r="23" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B23" s="25"/>
+      <c r="C23" s="21" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B18" s="33"/>
-      <c r="C18" s="40"/>
-      <c r="D18" s="2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="19" spans="2:4" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B19" s="33"/>
-      <c r="C19" s="41"/>
-      <c r="D19" s="4" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B20" s="33"/>
-      <c r="C20" s="15" t="s">
-        <v>137</v>
-      </c>
-      <c r="D20" s="2"/>
-    </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B21" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="C21" s="18" t="s">
-        <v>68</v>
-      </c>
-      <c r="D21" s="19"/>
-    </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B22" s="21"/>
-      <c r="C22" s="18" t="s">
-        <v>126</v>
-      </c>
-      <c r="D22" s="19"/>
-    </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B23" s="22"/>
-      <c r="C23" s="18" t="s">
-        <v>138</v>
-      </c>
-      <c r="D23" s="19"/>
+      <c r="D23" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="C16:C19"/>
+    <mergeCell ref="B11:B20"/>
+    <mergeCell ref="B21:B23"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="C13:C15"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="C10:D10"/>
@@ -1958,13 +1965,6 @@
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="C7:D7"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="C16:C19"/>
-    <mergeCell ref="B11:B20"/>
-    <mergeCell ref="B21:B23"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="C13:C15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1984,85 +1984,85 @@
       <c r="B2" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="30" t="s">
+      <c r="C2" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="D2" s="31"/>
+      <c r="D2" s="20"/>
     </row>
     <row r="3" spans="2:4" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="28" t="s">
-        <v>73</v>
-      </c>
-      <c r="D3" s="29"/>
+      <c r="C3" s="30" t="s">
+        <v>72</v>
+      </c>
+      <c r="D3" s="31"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="18" t="s">
-        <v>72</v>
-      </c>
-      <c r="D4" s="19"/>
+      <c r="C4" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="D4" s="22"/>
     </row>
     <row r="5" spans="2:4" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="28" t="s">
-        <v>75</v>
-      </c>
-      <c r="D5" s="29"/>
+      <c r="C5" s="30" t="s">
+        <v>74</v>
+      </c>
+      <c r="D5" s="31"/>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B6" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="18" t="s">
-        <v>71</v>
-      </c>
-      <c r="D6" s="19"/>
+      <c r="C6" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="D6" s="22"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B7" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="18" t="s">
-        <v>70</v>
-      </c>
-      <c r="D7" s="19"/>
+      <c r="C7" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="22"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B8" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="18" t="s">
-        <v>74</v>
-      </c>
-      <c r="D8" s="19"/>
+      <c r="C8" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="D8" s="22"/>
     </row>
     <row r="9" spans="2:4" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="28" t="s">
-        <v>76</v>
-      </c>
-      <c r="D9" s="29"/>
+      <c r="C9" s="30" t="s">
+        <v>75</v>
+      </c>
+      <c r="D9" s="31"/>
     </row>
     <row r="10" spans="2:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="28" t="s">
-        <v>77</v>
-      </c>
-      <c r="D10" s="19"/>
+      <c r="C10" s="30" t="s">
+        <v>76</v>
+      </c>
+      <c r="D10" s="22"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B11" s="20" t="s">
+      <c r="B11" s="23" t="s">
         <v>9</v>
       </c>
       <c r="C11" s="13" t="s">
@@ -2073,68 +2073,68 @@
       </c>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B12" s="21"/>
+      <c r="B12" s="24"/>
       <c r="C12" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="D12" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="D12" s="14" t="s">
+    </row>
+    <row r="13" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B13" s="24"/>
+      <c r="C13" s="18" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B13" s="21"/>
-      <c r="C13" s="47" t="s">
+      <c r="D13" s="14" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="14" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B14" s="24"/>
+      <c r="C14" s="28" t="s">
+        <v>135</v>
+      </c>
+      <c r="D14" s="14" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B15" s="24"/>
+      <c r="C15" s="29"/>
+      <c r="D15" s="14" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="24"/>
+      <c r="C16" s="32"/>
+      <c r="D16" s="6" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B17" s="25"/>
+      <c r="C17" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="D17" s="14"/>
+    </row>
+    <row r="18" spans="2:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="D13" s="14" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B14" s="21"/>
-      <c r="C14" s="25" t="s">
-        <v>139</v>
-      </c>
-      <c r="D14" s="14" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="15" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B15" s="21"/>
-      <c r="C15" s="26"/>
-      <c r="D15" s="14" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="16" spans="2:4" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="21"/>
-      <c r="C16" s="27"/>
-      <c r="D16" s="6" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B17" s="22"/>
-      <c r="C17" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="D17" s="14"/>
-    </row>
-    <row r="18" spans="2:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="C18" s="18" t="s">
-        <v>81</v>
-      </c>
-      <c r="D18" s="19"/>
+      <c r="D18" s="22"/>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B19" s="22"/>
-      <c r="C19" s="18" t="s">
-        <v>126</v>
-      </c>
-      <c r="D19" s="19"/>
+      <c r="B19" s="25"/>
+      <c r="C19" s="21" t="s">
+        <v>122</v>
+      </c>
+      <c r="D19" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -2171,85 +2171,85 @@
       <c r="B2" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="30" t="s">
-        <v>82</v>
-      </c>
-      <c r="D2" s="31"/>
+      <c r="C2" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="D2" s="20"/>
     </row>
     <row r="3" spans="2:4" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="28" t="s">
-        <v>84</v>
-      </c>
-      <c r="D3" s="29"/>
+      <c r="C3" s="30" t="s">
+        <v>83</v>
+      </c>
+      <c r="D3" s="31"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="18" t="s">
-        <v>85</v>
-      </c>
-      <c r="D4" s="19"/>
+      <c r="C4" s="21" t="s">
+        <v>84</v>
+      </c>
+      <c r="D4" s="22"/>
     </row>
     <row r="5" spans="2:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="28" t="s">
-        <v>86</v>
-      </c>
-      <c r="D5" s="29"/>
+      <c r="C5" s="30" t="s">
+        <v>85</v>
+      </c>
+      <c r="D5" s="31"/>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B6" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="18" t="s">
-        <v>71</v>
-      </c>
-      <c r="D6" s="19"/>
+      <c r="C6" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="D6" s="22"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B7" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="18" t="s">
-        <v>83</v>
-      </c>
-      <c r="D7" s="19"/>
+      <c r="C7" s="21" t="s">
+        <v>82</v>
+      </c>
+      <c r="D7" s="22"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B8" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="18" t="s">
-        <v>87</v>
-      </c>
-      <c r="D8" s="19"/>
+      <c r="C8" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D8" s="22"/>
     </row>
     <row r="9" spans="2:4" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="28" t="s">
-        <v>88</v>
-      </c>
-      <c r="D9" s="29"/>
+      <c r="C9" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="D9" s="31"/>
     </row>
     <row r="10" spans="2:4" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="28" t="s">
-        <v>89</v>
-      </c>
-      <c r="D10" s="19"/>
+      <c r="C10" s="30" t="s">
+        <v>88</v>
+      </c>
+      <c r="D10" s="22"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B11" s="20" t="s">
+      <c r="B11" s="23" t="s">
         <v>9</v>
       </c>
       <c r="C11" s="13" t="s">
@@ -2260,69 +2260,73 @@
       </c>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B12" s="21"/>
-      <c r="C12" s="48" t="s">
+      <c r="B12" s="24"/>
+      <c r="C12" s="44" t="s">
+        <v>89</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>91</v>
-      </c>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B13" s="21"/>
-      <c r="C13" s="49"/>
+      <c r="B13" s="24"/>
+      <c r="C13" s="45"/>
       <c r="D13" s="2" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B14" s="21"/>
-      <c r="C14" s="50"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="46"/>
       <c r="D14" s="2" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B15" s="21"/>
-      <c r="C15" s="25" t="s">
-        <v>92</v>
+      <c r="B15" s="24"/>
+      <c r="C15" s="28" t="s">
+        <v>157</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>93</v>
+        <v>155</v>
       </c>
     </row>
     <row r="16" spans="2:4" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B16" s="21"/>
-      <c r="C16" s="27"/>
+      <c r="B16" s="24"/>
+      <c r="C16" s="32"/>
       <c r="D16" s="4" t="s">
-        <v>94</v>
+        <v>156</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B17" s="22"/>
+      <c r="B17" s="25"/>
       <c r="C17" s="4" t="s">
-        <v>95</v>
+        <v>158</v>
       </c>
       <c r="D17" s="3"/>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B18" s="33" t="s">
+      <c r="B18" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="C18" s="32" t="s">
-        <v>81</v>
-      </c>
-      <c r="D18" s="32"/>
+      <c r="C18" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="D18" s="34"/>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B19" s="33"/>
-      <c r="C19" s="42" t="s">
-        <v>151</v>
-      </c>
-      <c r="D19" s="42"/>
+      <c r="B19" s="43"/>
+      <c r="C19" s="47" t="s">
+        <v>147</v>
+      </c>
+      <c r="D19" s="47"/>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="B11:B17"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="B18:B19"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="C10:D10"/>
@@ -2334,10 +2338,6 @@
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="C12:C14"/>
-    <mergeCell ref="B11:B17"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="B18:B19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2357,85 +2357,85 @@
       <c r="B2" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="30" t="s">
-        <v>96</v>
-      </c>
-      <c r="D2" s="31"/>
+      <c r="C2" s="19" t="s">
+        <v>92</v>
+      </c>
+      <c r="D2" s="20"/>
     </row>
     <row r="3" spans="2:4" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="28" t="s">
-        <v>98</v>
-      </c>
-      <c r="D3" s="29"/>
+      <c r="C3" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="D3" s="31"/>
     </row>
     <row r="4" spans="2:4" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="28" t="s">
-        <v>102</v>
-      </c>
-      <c r="D4" s="19"/>
+      <c r="C4" s="30" t="s">
+        <v>98</v>
+      </c>
+      <c r="D4" s="22"/>
     </row>
     <row r="5" spans="2:4" ht="50.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="28" t="s">
-        <v>99</v>
-      </c>
-      <c r="D5" s="29"/>
+      <c r="C5" s="30" t="s">
+        <v>95</v>
+      </c>
+      <c r="D5" s="31"/>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B6" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="19"/>
+      <c r="D6" s="22"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B7" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="19"/>
+      <c r="D7" s="22"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B8" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="D8" s="19"/>
+      <c r="D8" s="22"/>
     </row>
     <row r="9" spans="2:4" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="28" t="s">
-        <v>100</v>
-      </c>
-      <c r="D9" s="29"/>
+      <c r="C9" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="D9" s="31"/>
     </row>
     <row r="10" spans="2:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="28" t="s">
-        <v>101</v>
-      </c>
-      <c r="D10" s="19"/>
+      <c r="C10" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="D10" s="22"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B11" s="20" t="s">
+      <c r="B11" s="23" t="s">
         <v>9</v>
       </c>
       <c r="C11" s="13" t="s">
@@ -2446,61 +2446,61 @@
       </c>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B12" s="21"/>
+      <c r="B12" s="24"/>
       <c r="C12" s="2" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="D12" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B13" s="24"/>
+      <c r="C13" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="14" spans="2:4" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="24"/>
+      <c r="C14" s="28" t="s">
+        <v>144</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="24"/>
+      <c r="C15" s="29"/>
+      <c r="D15" s="2" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B13" s="21"/>
-      <c r="C13" s="4" t="s">
+    <row r="16" spans="2:4" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="25"/>
+      <c r="C16" s="32"/>
+      <c r="D16" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="D13" s="3" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="14" spans="2:4" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="21"/>
-      <c r="C14" s="25" t="s">
-        <v>148</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="15" spans="2:4" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="21"/>
-      <c r="C15" s="26"/>
-      <c r="D15" s="2" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="16" spans="2:4" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="22"/>
-      <c r="C16" s="27"/>
-      <c r="D16" s="4" t="s">
-        <v>150</v>
-      </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B17" s="20" t="s">
+      <c r="B17" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="23" t="s">
-        <v>117</v>
-      </c>
-      <c r="D17" s="24"/>
+      <c r="C17" s="26" t="s">
+        <v>113</v>
+      </c>
+      <c r="D17" s="27"/>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B18" s="22"/>
-      <c r="C18" s="32" t="s">
-        <v>126</v>
-      </c>
-      <c r="D18" s="32"/>
+      <c r="B18" s="25"/>
+      <c r="C18" s="34" t="s">
+        <v>122</v>
+      </c>
+      <c r="D18" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -2537,85 +2537,85 @@
       <c r="B2" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="30" t="s">
-        <v>97</v>
-      </c>
-      <c r="D2" s="31"/>
+      <c r="C2" s="19" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2" s="20"/>
     </row>
     <row r="3" spans="2:4" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="28" t="s">
-        <v>104</v>
-      </c>
-      <c r="D3" s="29"/>
+      <c r="C3" s="30" t="s">
+        <v>100</v>
+      </c>
+      <c r="D3" s="31"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="18" t="s">
-        <v>105</v>
-      </c>
-      <c r="D4" s="19"/>
+      <c r="C4" s="21" t="s">
+        <v>101</v>
+      </c>
+      <c r="D4" s="22"/>
     </row>
     <row r="5" spans="2:4" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="28" t="s">
-        <v>106</v>
-      </c>
-      <c r="D5" s="29"/>
+      <c r="C5" s="30" t="s">
+        <v>102</v>
+      </c>
+      <c r="D5" s="31"/>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B6" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="19"/>
+      <c r="D6" s="22"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B7" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="19"/>
+      <c r="D7" s="22"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B8" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="18" t="s">
-        <v>108</v>
-      </c>
-      <c r="D8" s="19"/>
+      <c r="C8" s="21" t="s">
+        <v>104</v>
+      </c>
+      <c r="D8" s="22"/>
     </row>
     <row r="9" spans="2:4" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="28" t="s">
-        <v>109</v>
-      </c>
-      <c r="D9" s="29"/>
+      <c r="C9" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="D9" s="31"/>
     </row>
     <row r="10" spans="2:4" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="28" t="s">
-        <v>110</v>
-      </c>
-      <c r="D10" s="19"/>
+      <c r="C10" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="D10" s="22"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B11" s="20" t="s">
+      <c r="B11" s="23" t="s">
         <v>9</v>
       </c>
       <c r="C11" s="13" t="s">
@@ -2626,99 +2626,104 @@
       </c>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B12" s="21"/>
+      <c r="B12" s="24"/>
       <c r="C12" s="2" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B13" s="21"/>
-      <c r="C13" s="25" t="s">
-        <v>112</v>
+      <c r="B13" s="24"/>
+      <c r="C13" s="28" t="s">
+        <v>108</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B14" s="21"/>
-      <c r="C14" s="26"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="29"/>
       <c r="D14" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="21"/>
-      <c r="C15" s="27"/>
+      <c r="B15" s="24"/>
+      <c r="C15" s="32"/>
       <c r="D15" s="2" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="24"/>
+      <c r="C16" s="28" t="s">
+        <v>150</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B17" s="24"/>
+      <c r="C17" s="29"/>
+      <c r="D17" s="2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B18" s="24"/>
+      <c r="C18" s="29"/>
+      <c r="D18" s="2" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="B19" s="24"/>
+      <c r="C19" s="32"/>
+      <c r="D19" s="4" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="16" spans="2:4" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="21"/>
-      <c r="C16" s="25" t="s">
-        <v>154</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B17" s="21"/>
-      <c r="C17" s="26"/>
-      <c r="D17" s="2" t="s">
+    <row r="20" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B20" s="25"/>
+      <c r="C20" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D20" s="3"/>
+    </row>
+    <row r="21" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B21" s="43" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="D21" s="34"/>
+    </row>
+    <row r="22" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B22" s="43"/>
+      <c r="C22" s="47" t="s">
+        <v>122</v>
+      </c>
+      <c r="D22" s="47"/>
+    </row>
+    <row r="23" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B23" s="43"/>
+      <c r="C23" s="47" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B18" s="21"/>
-      <c r="C18" s="26"/>
-      <c r="D18" s="2" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="19" spans="2:4" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B19" s="21"/>
-      <c r="C19" s="27"/>
-      <c r="D19" s="4" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B20" s="22"/>
-      <c r="C20" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="D20" s="3"/>
-    </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B21" s="33" t="s">
-        <v>12</v>
-      </c>
-      <c r="C21" s="32" t="s">
-        <v>28</v>
-      </c>
-      <c r="D21" s="32"/>
-    </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B22" s="33"/>
-      <c r="C22" s="42" t="s">
-        <v>126</v>
-      </c>
-      <c r="D22" s="42"/>
-    </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B23" s="33"/>
-      <c r="C23" s="42" t="s">
-        <v>157</v>
-      </c>
-      <c r="D23" s="42"/>
+      <c r="D23" s="47"/>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C6:D6"/>
     <mergeCell ref="B21:B23"/>
     <mergeCell ref="C22:D22"/>
     <mergeCell ref="C23:D23"/>
@@ -2726,11 +2731,6 @@
     <mergeCell ref="C13:C15"/>
     <mergeCell ref="C16:C19"/>
     <mergeCell ref="B11:B20"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C6:D6"/>
     <mergeCell ref="C21:D21"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="C9:D9"/>
@@ -2754,69 +2754,69 @@
       <c r="B2" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="30"/>
-      <c r="D2" s="31"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="20"/>
     </row>
     <row r="3" spans="2:4" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="28"/>
-      <c r="D3" s="29"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="31"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="18"/>
-      <c r="D4" s="19"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="22"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B5" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="28"/>
-      <c r="D5" s="29"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="31"/>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B6" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="18"/>
-      <c r="D6" s="19"/>
+      <c r="C6" s="21"/>
+      <c r="D6" s="22"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B7" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="18"/>
-      <c r="D7" s="19"/>
+      <c r="C7" s="21"/>
+      <c r="D7" s="22"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B8" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="19"/>
+      <c r="D8" s="22"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B9" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="28"/>
-      <c r="D9" s="29"/>
+      <c r="C9" s="30"/>
+      <c r="D9" s="31"/>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B10" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="18"/>
-      <c r="D10" s="19"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="22"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B11" s="34" t="s">
+      <c r="B11" s="37" t="s">
         <v>9</v>
       </c>
       <c r="C11" s="13" t="s">
@@ -2827,65 +2827,59 @@
       </c>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B12" s="35"/>
+      <c r="B12" s="38"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B13" s="35"/>
+      <c r="B13" s="38"/>
       <c r="C13" s="4"/>
       <c r="D13" s="2"/>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B14" s="35"/>
+      <c r="B14" s="38"/>
       <c r="C14" s="4"/>
       <c r="D14" s="2"/>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B15" s="35"/>
+      <c r="B15" s="38"/>
       <c r="C15" s="4"/>
       <c r="D15" s="2"/>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B16" s="36"/>
+      <c r="B16" s="39"/>
       <c r="C16" s="4"/>
       <c r="D16" s="2"/>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B17" s="44" t="s">
+      <c r="B17" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="18"/>
-      <c r="D17" s="19"/>
+      <c r="C17" s="21"/>
+      <c r="D17" s="22"/>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B18" s="44"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="19"/>
+      <c r="B18" s="48"/>
+      <c r="C18" s="21"/>
+      <c r="D18" s="22"/>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B19" s="44"/>
-      <c r="C19" s="18"/>
-      <c r="D19" s="19"/>
+      <c r="B19" s="48"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="22"/>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B20" s="44"/>
-      <c r="C20" s="45"/>
-      <c r="D20" s="46"/>
+      <c r="B20" s="48"/>
+      <c r="C20" s="49"/>
+      <c r="D20" s="50"/>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B21" s="44"/>
-      <c r="C21" s="32"/>
-      <c r="D21" s="32"/>
+      <c r="B21" s="48"/>
+      <c r="C21" s="34"/>
+      <c r="D21" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C6:D6"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="C10:D10"/>
@@ -2896,6 +2890,12 @@
     <mergeCell ref="C19:D19"/>
     <mergeCell ref="C20:D20"/>
     <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C6:D6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>